<commit_message>
chore: repository cleanup, environment template, and test suite configuration
</commit_message>
<xml_diff>
--- a/load-tests/DevPrep_AI_Load_Test_Report.xlsx
+++ b/load-tests/DevPrep_AI_Load_Test_Report.xlsx
@@ -53,7 +53,7 @@
     <t>Requests Per Second (RPS)</t>
   </si>
   <si>
-    <t>474.84 req/sec</t>
+    <t>446.08 req/sec</t>
   </si>
   <si>
     <t>Total Executed Requests</t>
@@ -65,37 +65,37 @@
     <t>Minimum Latency</t>
   </si>
   <si>
-    <t>104 ms</t>
+    <t>128 ms</t>
   </si>
   <si>
     <t>Average Latency</t>
   </si>
   <si>
-    <t>199.77 ms</t>
+    <t>214.13 ms</t>
   </si>
   <si>
     <t>p50 Latency</t>
   </si>
   <si>
-    <t>195 ms</t>
+    <t>204 ms</t>
   </si>
   <si>
     <t>p95 Latency</t>
   </si>
   <si>
-    <t>259 ms</t>
+    <t>275 ms</t>
   </si>
   <si>
     <t>p99 Latency</t>
   </si>
   <si>
-    <t>289 ms</t>
+    <t>315 ms</t>
   </si>
   <si>
     <t>Maximum Latency</t>
   </si>
   <si>
-    <t>307 ms</t>
+    <t>333 ms</t>
   </si>
   <si>
     <t>Responses</t>
@@ -134,7 +134,7 @@
     <t>Transfer Speed (MB/sec)</t>
   </si>
   <si>
-    <t>0.59 MB/sec</t>
+    <t>0.55 MB/sec</t>
   </si>
   <si>
     <t>Evaluation</t>
@@ -642,7 +642,7 @@
         <v>14</v>
       </c>
       <c r="C7">
-        <v>1453</v>
+        <v>1365</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
@@ -719,7 +719,7 @@
         <v>29</v>
       </c>
       <c r="C14">
-        <v>1453</v>
+        <v>1365</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
@@ -849,7 +849,7 @@
         <v>49</v>
       </c>
       <c r="C2">
-        <v>1453</v>
+        <v>1365</v>
       </c>
       <c r="D2" t="s">
         <v>35</v>

</xml_diff>